<commit_message>
add new column employee id
</commit_message>
<xml_diff>
--- a/src/assets/bulkuser_excel_sheet.xlsx
+++ b/src/assets/bulkuser_excel_sheet.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Saurav Mishra\Downloads\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B0BBFD4-04DB-4FD9-9F23-42632F817F08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="19160" windowHeight="6350"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bulk User" sheetId="1" r:id="rId1"/>
@@ -29,8 +35,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -38,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="160">
   <si>
     <t>Title</t>
   </si>
@@ -516,20 +520,19 @@
   </si>
   <si>
     <t>test_UAT</t>
+  </si>
+  <si>
+    <t>EmployeeId</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="5">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="178" formatCode="[$-14009]yyyy/mm/dd;@"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="166" formatCode="[$-14009]yyyy/mm/dd;@"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -580,151 +583,8 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="34">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -737,194 +597,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="9">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -932,249 +606,10 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1186,71 +621,28 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="178" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="6" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1508,43 +900,43 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:AD2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelRow="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:AE2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="14.5" customWidth="1"/>
+    <col min="1" max="1" width="14.44140625" customWidth="1"/>
     <col min="2" max="2" width="19" customWidth="1"/>
-    <col min="3" max="3" width="23.1272727272727" customWidth="1"/>
-    <col min="4" max="4" width="20.7545454545455" customWidth="1"/>
-    <col min="5" max="5" width="17.1272727272727" customWidth="1"/>
-    <col min="6" max="6" width="22.5" style="4" customWidth="1"/>
-    <col min="7" max="7" width="19.3727272727273" customWidth="1"/>
-    <col min="8" max="8" width="32.2545454545455" style="4" customWidth="1"/>
-    <col min="9" max="9" width="21.1272727272727" style="5" customWidth="1"/>
-    <col min="10" max="10" width="9.12727272727273" style="4" customWidth="1"/>
-    <col min="11" max="13" width="25.3727272727273" customWidth="1"/>
-    <col min="14" max="14" width="24" customWidth="1"/>
-    <col min="15" max="15" width="24.7545454545455" style="4" customWidth="1"/>
-    <col min="16" max="16" width="11.8727272727273" customWidth="1"/>
-    <col min="17" max="17" width="20.6272727272727" customWidth="1"/>
-    <col min="18" max="18" width="20.1272727272727" customWidth="1"/>
-    <col min="19" max="19" width="20.7545454545455" customWidth="1"/>
-    <col min="20" max="20" width="20.3727272727273" customWidth="1"/>
-    <col min="21" max="21" width="16.7545454545455" customWidth="1"/>
-    <col min="22" max="24" width="28.8727272727273" customWidth="1"/>
-    <col min="25" max="25" width="21.6272727272727" style="4" customWidth="1"/>
-    <col min="26" max="26" width="35.6272727272727" customWidth="1"/>
-    <col min="27" max="28" width="28.8727272727273" customWidth="1"/>
-    <col min="29" max="29" width="28.8727272727273" style="4" customWidth="1"/>
-    <col min="30" max="30" width="21.1272727272727" style="5" customWidth="1"/>
+    <col min="3" max="3" width="23.109375" customWidth="1"/>
+    <col min="4" max="4" width="20.77734375" customWidth="1"/>
+    <col min="5" max="5" width="17.109375" customWidth="1"/>
+    <col min="6" max="6" width="22.44140625" style="4" customWidth="1"/>
+    <col min="7" max="7" width="19.33203125" customWidth="1"/>
+    <col min="8" max="8" width="32.21875" style="4" customWidth="1"/>
+    <col min="9" max="9" width="21.109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="9.109375" style="4" customWidth="1"/>
+    <col min="11" max="14" width="25.33203125" customWidth="1"/>
+    <col min="15" max="15" width="24" customWidth="1"/>
+    <col min="16" max="16" width="24.77734375" style="4" customWidth="1"/>
+    <col min="17" max="17" width="11.88671875" customWidth="1"/>
+    <col min="18" max="18" width="20.6640625" customWidth="1"/>
+    <col min="19" max="19" width="20.109375" customWidth="1"/>
+    <col min="20" max="20" width="20.77734375" customWidth="1"/>
+    <col min="21" max="21" width="20.33203125" customWidth="1"/>
+    <col min="22" max="22" width="16.77734375" customWidth="1"/>
+    <col min="23" max="25" width="28.88671875" customWidth="1"/>
+    <col min="26" max="26" width="21.6640625" style="4" customWidth="1"/>
+    <col min="27" max="27" width="35.6640625" customWidth="1"/>
+    <col min="28" max="29" width="28.88671875" customWidth="1"/>
+    <col min="30" max="30" width="28.88671875" style="4" customWidth="1"/>
+    <col min="31" max="31" width="21.109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="3" customFormat="1" ht="23.5" spans="1:30">
+    <row r="1" spans="1:31" s="3" customFormat="1" ht="23.4">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -1584,110 +976,139 @@
       <c r="M1" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="7" t="s">
+      <c r="N1" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="O1" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="11" t="s">
+      <c r="P1" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="7" t="s">
+      <c r="Q1" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="6" t="s">
+      <c r="R1" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="7" t="s">
+      <c r="S1" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="7" t="s">
+      <c r="T1" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="7" t="s">
+      <c r="U1" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="7" t="s">
+      <c r="V1" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="7" t="s">
+      <c r="W1" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="6" t="s">
+      <c r="X1" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="6" t="s">
+      <c r="Y1" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="11" t="s">
+      <c r="Z1" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="7" t="s">
+      <c r="AA1" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="6" t="s">
+      <c r="AB1" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="13" t="s">
+      <c r="AC1" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="11" t="s">
+      <c r="AD1" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="9" t="s">
+      <c r="AE1" s="9" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="11:11">
+    <row r="2" spans="1:31">
       <c r="K2" s="12"/>
     </row>
   </sheetData>
-  <dataValidations count="8">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A1048576">
-      <formula1>Help!$C$2:$C$7</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E1048576">
-      <formula1>Help!$B$1:$B$5</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1048576">
-      <formula1>Help!$D$2:$D$50</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2:N1048576">
-      <formula1>Help!$E$2:$E$8</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q2:Q1048576">
-      <formula1>Help!$F$2:$F$6</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T$1:T$1048576">
-      <formula1>Help!$G$2:$G$9</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U2:U1048576">
-      <formula1>Help!$H$2:$H$9</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="W2:W1048576 AA2:AA1048576">
-      <formula1>Help!$I$2:$I$38</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="8">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000000000000}">
+          <x14:formula1>
+            <xm:f>Help!$C$2:$C$7</xm:f>
+          </x14:formula1>
+          <xm:sqref>A2:A1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000001000000}">
+          <x14:formula1>
+            <xm:f>Help!$B$1:$B$5</xm:f>
+          </x14:formula1>
+          <xm:sqref>E2:E1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
+          <x14:formula1>
+            <xm:f>Help!$D$2:$D$50</xm:f>
+          </x14:formula1>
+          <xm:sqref>G2:G1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000003000000}">
+          <x14:formula1>
+            <xm:f>Help!$E$2:$E$8</xm:f>
+          </x14:formula1>
+          <xm:sqref>O2:O1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000004000000}">
+          <x14:formula1>
+            <xm:f>Help!$F$2:$F$6</xm:f>
+          </x14:formula1>
+          <xm:sqref>R2:R1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000005000000}">
+          <x14:formula1>
+            <xm:f>Help!$G$2:$G$9</xm:f>
+          </x14:formula1>
+          <xm:sqref>U1:U1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000006000000}">
+          <x14:formula1>
+            <xm:f>Help!$H$2:$H$9</xm:f>
+          </x14:formula1>
+          <xm:sqref>V2:V1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000007000000}">
+          <x14:formula1>
+            <xm:f>Help!$I$2:$I$38</xm:f>
+          </x14:formula1>
+          <xm:sqref>X2:X1048576 AB2:AB1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I50"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="17.5" customWidth="1"/>
-    <col min="2" max="2" width="16.1272727272727" style="1" customWidth="1"/>
-    <col min="3" max="3" width="8.87272727272727" style="1"/>
-    <col min="4" max="4" width="32.6272727272727" customWidth="1"/>
-    <col min="5" max="5" width="13.6272727272727" customWidth="1"/>
-    <col min="6" max="6" width="19.5" customWidth="1"/>
-    <col min="7" max="7" width="13.5" customWidth="1"/>
-    <col min="8" max="8" width="13.7545454545455" customWidth="1"/>
-    <col min="9" max="9" width="27.1272727272727" customWidth="1"/>
-    <col min="12" max="12" width="8.87272727272727" customWidth="1"/>
+    <col min="1" max="1" width="17.44140625" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8.88671875" style="1"/>
+    <col min="4" max="4" width="32.6640625" customWidth="1"/>
+    <col min="5" max="5" width="13.6640625" customWidth="1"/>
+    <col min="6" max="6" width="19.44140625" customWidth="1"/>
+    <col min="7" max="7" width="13.44140625" customWidth="1"/>
+    <col min="8" max="8" width="13.77734375" customWidth="1"/>
+    <col min="9" max="9" width="27.109375" customWidth="1"/>
+    <col min="12" max="12" width="8.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -1777,7 +1198,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="4" ht="15.6" customHeight="1" spans="1:9">
+    <row r="4" spans="1:9" ht="15.6" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>49</v>
       </c>
@@ -1904,7 +1325,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="9" spans="4:9">
+    <row r="9" spans="1:9">
       <c r="D9" t="s">
         <v>84</v>
       </c>
@@ -1918,7 +1339,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="10" spans="4:9">
+    <row r="10" spans="1:9">
       <c r="D10" t="s">
         <v>88</v>
       </c>
@@ -1929,7 +1350,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="4:9">
+    <row r="11" spans="1:9">
       <c r="D11" t="s">
         <v>91</v>
       </c>
@@ -1937,7 +1358,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="12" spans="4:9">
+    <row r="12" spans="1:9">
       <c r="D12" t="s">
         <v>93</v>
       </c>
@@ -1945,7 +1366,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="13" spans="4:9">
+    <row r="13" spans="1:9">
       <c r="D13" t="s">
         <v>95</v>
       </c>
@@ -1953,7 +1374,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="14" spans="4:9">
+    <row r="14" spans="1:9">
       <c r="D14" t="s">
         <v>97</v>
       </c>
@@ -1961,7 +1382,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="15" spans="4:9">
+    <row r="15" spans="1:9">
       <c r="D15" t="s">
         <v>99</v>
       </c>
@@ -1969,7 +1390,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="16" spans="4:9">
+    <row r="16" spans="1:9">
       <c r="D16" t="s">
         <v>101</v>
       </c>
@@ -2153,52 +1574,52 @@
         <v>146</v>
       </c>
     </row>
-    <row r="39" spans="4:4">
+    <row r="39" spans="4:9">
       <c r="D39" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="40" spans="4:4">
+    <row r="40" spans="4:9">
       <c r="D40" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="41" spans="4:4">
+    <row r="41" spans="4:9">
       <c r="D41" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="42" spans="4:4">
+    <row r="42" spans="4:9">
       <c r="D42" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="43" spans="4:4">
+    <row r="43" spans="4:9">
       <c r="D43" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="44" spans="4:4">
+    <row r="44" spans="4:9">
       <c r="D44" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="45" spans="4:4">
+    <row r="45" spans="4:9">
       <c r="D45" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="46" spans="4:4">
+    <row r="46" spans="4:9">
       <c r="D46" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="47" spans="4:4">
+    <row r="47" spans="4:9">
       <c r="D47" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="48" spans="4:4">
+    <row r="48" spans="4:9">
       <c r="D48" t="s">
         <v>156</v>
       </c>
@@ -2215,7 +1636,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix/employee id column (#164)
* add new column employee id

* add new column employee id
</commit_message>
<xml_diff>
--- a/src/assets/bulkuser_excel_sheet.xlsx
+++ b/src/assets/bulkuser_excel_sheet.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Saurav Mishra\Downloads\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEAC646A-623A-49D9-8CFC-12A95AC02EFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="19160" windowHeight="6350"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bulk User" sheetId="1" r:id="rId1"/>
@@ -29,8 +35,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -38,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="160">
   <si>
     <t>Title</t>
   </si>
@@ -516,20 +520,19 @@
   </si>
   <si>
     <t>test_UAT</t>
+  </si>
+  <si>
+    <t>EmployeeId</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="5">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="178" formatCode="[$-14009]yyyy/mm/dd;@"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="166" formatCode="[$-14009]yyyy/mm/dd;@"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -565,14 +568,6 @@
       <charset val="134"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="18"/>
       <color rgb="FFFF0000"/>
@@ -580,151 +575,8 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="34">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -737,194 +589,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="9">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -932,253 +598,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1186,71 +610,26 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="178" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="6" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1508,43 +887,44 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:AD2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelRow="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:AE1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="14.5" customWidth="1"/>
+    <col min="1" max="1" width="14.44140625" customWidth="1"/>
     <col min="2" max="2" width="19" customWidth="1"/>
-    <col min="3" max="3" width="23.1272727272727" customWidth="1"/>
-    <col min="4" max="4" width="20.7545454545455" customWidth="1"/>
-    <col min="5" max="5" width="17.1272727272727" customWidth="1"/>
-    <col min="6" max="6" width="22.5" style="4" customWidth="1"/>
-    <col min="7" max="7" width="19.3727272727273" customWidth="1"/>
-    <col min="8" max="8" width="32.2545454545455" style="4" customWidth="1"/>
-    <col min="9" max="9" width="21.1272727272727" style="5" customWidth="1"/>
-    <col min="10" max="10" width="9.12727272727273" style="4" customWidth="1"/>
-    <col min="11" max="13" width="25.3727272727273" customWidth="1"/>
-    <col min="14" max="14" width="24" customWidth="1"/>
-    <col min="15" max="15" width="24.7545454545455" style="4" customWidth="1"/>
-    <col min="16" max="16" width="11.8727272727273" customWidth="1"/>
-    <col min="17" max="17" width="20.6272727272727" customWidth="1"/>
-    <col min="18" max="18" width="20.1272727272727" customWidth="1"/>
-    <col min="19" max="19" width="20.7545454545455" customWidth="1"/>
-    <col min="20" max="20" width="20.3727272727273" customWidth="1"/>
-    <col min="21" max="21" width="16.7545454545455" customWidth="1"/>
-    <col min="22" max="24" width="28.8727272727273" customWidth="1"/>
-    <col min="25" max="25" width="21.6272727272727" style="4" customWidth="1"/>
-    <col min="26" max="26" width="35.6272727272727" customWidth="1"/>
-    <col min="27" max="28" width="28.8727272727273" customWidth="1"/>
-    <col min="29" max="29" width="28.8727272727273" style="4" customWidth="1"/>
-    <col min="30" max="30" width="21.1272727272727" style="5" customWidth="1"/>
+    <col min="3" max="3" width="23.109375" customWidth="1"/>
+    <col min="4" max="4" width="20.77734375" customWidth="1"/>
+    <col min="5" max="5" width="17.109375" customWidth="1"/>
+    <col min="6" max="6" width="22.44140625" style="4" customWidth="1"/>
+    <col min="7" max="7" width="19.33203125" customWidth="1"/>
+    <col min="8" max="8" width="32.21875" style="4" customWidth="1"/>
+    <col min="9" max="9" width="21.109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="9.109375" style="4" customWidth="1"/>
+    <col min="11" max="14" width="25.33203125" customWidth="1"/>
+    <col min="15" max="15" width="24" customWidth="1"/>
+    <col min="16" max="16" width="24.77734375" style="4" customWidth="1"/>
+    <col min="17" max="17" width="11.88671875" customWidth="1"/>
+    <col min="18" max="18" width="20.6640625" customWidth="1"/>
+    <col min="19" max="19" width="20.109375" customWidth="1"/>
+    <col min="20" max="20" width="20.77734375" customWidth="1"/>
+    <col min="21" max="21" width="20.33203125" customWidth="1"/>
+    <col min="22" max="22" width="16.77734375" customWidth="1"/>
+    <col min="23" max="23" width="32.21875" customWidth="1"/>
+    <col min="24" max="25" width="28.88671875" customWidth="1"/>
+    <col min="26" max="26" width="21.6640625" style="4" customWidth="1"/>
+    <col min="27" max="27" width="35.6640625" customWidth="1"/>
+    <col min="28" max="29" width="28.88671875" customWidth="1"/>
+    <col min="30" max="30" width="28.88671875" style="4" customWidth="1"/>
+    <col min="31" max="31" width="21.109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="3" customFormat="1" ht="23.5" spans="1:30">
+    <row r="1" spans="1:31" s="3" customFormat="1" ht="23.4">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -1584,110 +964,139 @@
       <c r="M1" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="7" t="s">
+      <c r="N1" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="O1" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="11" t="s">
+      <c r="P1" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="7" t="s">
+      <c r="Q1" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="6" t="s">
+      <c r="R1" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="7" t="s">
+      <c r="S1" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="7" t="s">
+      <c r="T1" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="7" t="s">
+      <c r="U1" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="7" t="s">
+      <c r="V1" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="7" t="s">
+      <c r="W1" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="6" t="s">
+      <c r="X1" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="6" t="s">
+      <c r="Y1" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="11" t="s">
+      <c r="Z1" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="7" t="s">
+      <c r="AA1" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="6" t="s">
+      <c r="AB1" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="13" t="s">
+      <c r="AC1" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="11" t="s">
+      <c r="AD1" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="9" t="s">
+      <c r="AE1" s="9" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="11:11">
-      <c r="K2" s="12"/>
-    </row>
   </sheetData>
-  <dataValidations count="8">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A1048576">
-      <formula1>Help!$C$2:$C$7</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E1048576">
-      <formula1>Help!$B$1:$B$5</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1048576">
-      <formula1>Help!$D$2:$D$50</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2:N1048576">
-      <formula1>Help!$E$2:$E$8</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q2:Q1048576">
-      <formula1>Help!$F$2:$F$6</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T$1:T$1048576">
-      <formula1>Help!$G$2:$G$9</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U2:U1048576">
-      <formula1>Help!$H$2:$H$9</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="W2:W1048576 AA2:AA1048576">
-      <formula1>Help!$I$2:$I$38</formula1>
-    </dataValidation>
+  <dataValidations count="1">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Date Format" prompt="YYYY-MM-DD" sqref="I1:I1048576 AE1:AE1048576" xr:uid="{87A554BA-43A4-4D4B-9158-4430D3C8FB3D}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="8">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000000000000}">
+          <x14:formula1>
+            <xm:f>Help!$C$2:$C$7</xm:f>
+          </x14:formula1>
+          <xm:sqref>A2:A1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000001000000}">
+          <x14:formula1>
+            <xm:f>Help!$B$1:$B$5</xm:f>
+          </x14:formula1>
+          <xm:sqref>E2:E1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
+          <x14:formula1>
+            <xm:f>Help!$D$2:$D$50</xm:f>
+          </x14:formula1>
+          <xm:sqref>G2:G1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000003000000}">
+          <x14:formula1>
+            <xm:f>Help!$E$2:$E$8</xm:f>
+          </x14:formula1>
+          <xm:sqref>O2:O1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000004000000}">
+          <x14:formula1>
+            <xm:f>Help!$F$2:$F$6</xm:f>
+          </x14:formula1>
+          <xm:sqref>R2:R1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000005000000}">
+          <x14:formula1>
+            <xm:f>Help!$G$2:$G$9</xm:f>
+          </x14:formula1>
+          <xm:sqref>U1:U1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000006000000}">
+          <x14:formula1>
+            <xm:f>Help!$H$2:$H$9</xm:f>
+          </x14:formula1>
+          <xm:sqref>V2:V1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000007000000}">
+          <x14:formula1>
+            <xm:f>Help!$I$2:$I$38</xm:f>
+          </x14:formula1>
+          <xm:sqref>AB2:AB1048576 X2:X1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I50"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="17.5" customWidth="1"/>
-    <col min="2" max="2" width="16.1272727272727" style="1" customWidth="1"/>
-    <col min="3" max="3" width="8.87272727272727" style="1"/>
-    <col min="4" max="4" width="32.6272727272727" customWidth="1"/>
-    <col min="5" max="5" width="13.6272727272727" customWidth="1"/>
-    <col min="6" max="6" width="19.5" customWidth="1"/>
-    <col min="7" max="7" width="13.5" customWidth="1"/>
-    <col min="8" max="8" width="13.7545454545455" customWidth="1"/>
-    <col min="9" max="9" width="27.1272727272727" customWidth="1"/>
-    <col min="12" max="12" width="8.87272727272727" customWidth="1"/>
+    <col min="1" max="1" width="17.44140625" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8.88671875" style="1"/>
+    <col min="4" max="4" width="32.6640625" customWidth="1"/>
+    <col min="5" max="5" width="13.6640625" customWidth="1"/>
+    <col min="6" max="6" width="19.44140625" customWidth="1"/>
+    <col min="7" max="7" width="13.44140625" customWidth="1"/>
+    <col min="8" max="8" width="13.77734375" customWidth="1"/>
+    <col min="9" max="9" width="27.109375" customWidth="1"/>
+    <col min="12" max="12" width="8.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -1777,7 +1186,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="4" ht="15.6" customHeight="1" spans="1:9">
+    <row r="4" spans="1:9" ht="15.6" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>49</v>
       </c>
@@ -1904,7 +1313,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="9" spans="4:9">
+    <row r="9" spans="1:9">
       <c r="D9" t="s">
         <v>84</v>
       </c>
@@ -1918,7 +1327,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="10" spans="4:9">
+    <row r="10" spans="1:9">
       <c r="D10" t="s">
         <v>88</v>
       </c>
@@ -1929,7 +1338,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="4:9">
+    <row r="11" spans="1:9">
       <c r="D11" t="s">
         <v>91</v>
       </c>
@@ -1937,7 +1346,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="12" spans="4:9">
+    <row r="12" spans="1:9">
       <c r="D12" t="s">
         <v>93</v>
       </c>
@@ -1945,7 +1354,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="13" spans="4:9">
+    <row r="13" spans="1:9">
       <c r="D13" t="s">
         <v>95</v>
       </c>
@@ -1953,7 +1362,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="14" spans="4:9">
+    <row r="14" spans="1:9">
       <c r="D14" t="s">
         <v>97</v>
       </c>
@@ -1961,7 +1370,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="15" spans="4:9">
+    <row r="15" spans="1:9">
       <c r="D15" t="s">
         <v>99</v>
       </c>
@@ -1969,7 +1378,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="16" spans="4:9">
+    <row r="16" spans="1:9">
       <c r="D16" t="s">
         <v>101</v>
       </c>
@@ -2153,52 +1562,52 @@
         <v>146</v>
       </c>
     </row>
-    <row r="39" spans="4:4">
+    <row r="39" spans="4:9">
       <c r="D39" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="40" spans="4:4">
+    <row r="40" spans="4:9">
       <c r="D40" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="41" spans="4:4">
+    <row r="41" spans="4:9">
       <c r="D41" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="42" spans="4:4">
+    <row r="42" spans="4:9">
       <c r="D42" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="43" spans="4:4">
+    <row r="43" spans="4:9">
       <c r="D43" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="44" spans="4:4">
+    <row r="44" spans="4:9">
       <c r="D44" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="45" spans="4:4">
+    <row r="45" spans="4:9">
       <c r="D45" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="46" spans="4:4">
+    <row r="46" spans="4:9">
       <c r="D46" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="47" spans="4:4">
+    <row r="47" spans="4:9">
       <c r="D47" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="48" spans="4:4">
+    <row r="48" spans="4:9">
       <c r="D48" t="s">
         <v>156</v>
       </c>
@@ -2215,7 +1624,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: keep the bulk user upload template from release-3.8.4
The release-3.11.0 merge brought a new bulkuser_excel_sheet.xlsx; this
branch keeps the 3.8.4 template.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/assets/bulkuser_excel_sheet.xlsx
+++ b/src/assets/bulkuser_excel_sheet.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Saurav Mishra\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEAC646A-623A-49D9-8CFC-12A95AC02EFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView windowWidth="19160" windowHeight="6350"/>
   </bookViews>
   <sheets>
     <sheet name="Bulk User" sheetId="1" r:id="rId1"/>
@@ -35,6 +29,8 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -42,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="159">
   <si>
     <t>Title</t>
   </si>
@@ -520,19 +516,20 @@
   </si>
   <si>
     <t>test_UAT</t>
-  </si>
-  <si>
-    <t>EmployeeId</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="[$-14009]yyyy/mm/dd;@"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="5">
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="178" formatCode="[$-14009]yyyy/mm/dd;@"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -568,6 +565,14 @@
       <charset val="134"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="18"/>
       <color rgb="FFFF0000"/>
@@ -575,8 +580,151 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -589,8 +737,194 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -598,11 +932,253 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="176" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -610,26 +1186,71 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="178" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="6" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -887,44 +1508,43 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AE1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:AD2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelRow="1"/>
   <cols>
-    <col min="1" max="1" width="14.44140625" customWidth="1"/>
+    <col min="1" max="1" width="14.5" customWidth="1"/>
     <col min="2" max="2" width="19" customWidth="1"/>
-    <col min="3" max="3" width="23.109375" customWidth="1"/>
-    <col min="4" max="4" width="20.77734375" customWidth="1"/>
-    <col min="5" max="5" width="17.109375" customWidth="1"/>
-    <col min="6" max="6" width="22.44140625" style="4" customWidth="1"/>
-    <col min="7" max="7" width="19.33203125" customWidth="1"/>
-    <col min="8" max="8" width="32.21875" style="4" customWidth="1"/>
-    <col min="9" max="9" width="21.109375" style="5" customWidth="1"/>
-    <col min="10" max="10" width="9.109375" style="4" customWidth="1"/>
-    <col min="11" max="14" width="25.33203125" customWidth="1"/>
-    <col min="15" max="15" width="24" customWidth="1"/>
-    <col min="16" max="16" width="24.77734375" style="4" customWidth="1"/>
-    <col min="17" max="17" width="11.88671875" customWidth="1"/>
-    <col min="18" max="18" width="20.6640625" customWidth="1"/>
-    <col min="19" max="19" width="20.109375" customWidth="1"/>
-    <col min="20" max="20" width="20.77734375" customWidth="1"/>
-    <col min="21" max="21" width="20.33203125" customWidth="1"/>
-    <col min="22" max="22" width="16.77734375" customWidth="1"/>
-    <col min="23" max="23" width="32.21875" customWidth="1"/>
-    <col min="24" max="25" width="28.88671875" customWidth="1"/>
-    <col min="26" max="26" width="21.6640625" style="4" customWidth="1"/>
-    <col min="27" max="27" width="35.6640625" customWidth="1"/>
-    <col min="28" max="29" width="28.88671875" customWidth="1"/>
-    <col min="30" max="30" width="28.88671875" style="4" customWidth="1"/>
-    <col min="31" max="31" width="21.109375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="23.1272727272727" customWidth="1"/>
+    <col min="4" max="4" width="20.7545454545455" customWidth="1"/>
+    <col min="5" max="5" width="17.1272727272727" customWidth="1"/>
+    <col min="6" max="6" width="22.5" style="4" customWidth="1"/>
+    <col min="7" max="7" width="19.3727272727273" customWidth="1"/>
+    <col min="8" max="8" width="32.2545454545455" style="4" customWidth="1"/>
+    <col min="9" max="9" width="21.1272727272727" style="5" customWidth="1"/>
+    <col min="10" max="10" width="9.12727272727273" style="4" customWidth="1"/>
+    <col min="11" max="13" width="25.3727272727273" customWidth="1"/>
+    <col min="14" max="14" width="24" customWidth="1"/>
+    <col min="15" max="15" width="24.7545454545455" style="4" customWidth="1"/>
+    <col min="16" max="16" width="11.8727272727273" customWidth="1"/>
+    <col min="17" max="17" width="20.6272727272727" customWidth="1"/>
+    <col min="18" max="18" width="20.1272727272727" customWidth="1"/>
+    <col min="19" max="19" width="20.7545454545455" customWidth="1"/>
+    <col min="20" max="20" width="20.3727272727273" customWidth="1"/>
+    <col min="21" max="21" width="16.7545454545455" customWidth="1"/>
+    <col min="22" max="24" width="28.8727272727273" customWidth="1"/>
+    <col min="25" max="25" width="21.6272727272727" style="4" customWidth="1"/>
+    <col min="26" max="26" width="35.6272727272727" customWidth="1"/>
+    <col min="27" max="28" width="28.8727272727273" customWidth="1"/>
+    <col min="29" max="29" width="28.8727272727273" style="4" customWidth="1"/>
+    <col min="30" max="30" width="21.1272727272727" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" s="3" customFormat="1" ht="23.4">
+    <row r="1" s="3" customFormat="1" ht="23.5" spans="1:30">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -964,139 +1584,110 @@
       <c r="M1" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="O1" s="7" t="s">
+      <c r="N1" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="11" t="s">
+      <c r="O1" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" s="7" t="s">
+      <c r="P1" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="R1" s="6" t="s">
+      <c r="Q1" s="6" t="s">
         <v>16</v>
       </c>
+      <c r="R1" s="7" t="s">
+        <v>17</v>
+      </c>
       <c r="S1" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="T1" s="7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="U1" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="V1" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="W1" s="7" t="s">
         <v>21</v>
       </c>
+      <c r="W1" s="6" t="s">
+        <v>22</v>
+      </c>
       <c r="X1" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="Y1" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="Z1" s="11" t="s">
+      <c r="Y1" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="AA1" s="7" t="s">
+      <c r="Z1" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="AB1" s="6" t="s">
+      <c r="AA1" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="AC1" s="12" t="s">
+      <c r="AB1" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="AD1" s="11" t="s">
+      <c r="AC1" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="AE1" s="9" t="s">
+      <c r="AD1" s="9" t="s">
         <v>29</v>
       </c>
     </row>
+    <row r="2" spans="11:11">
+      <c r="K2" s="12"/>
+    </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Date Format" prompt="YYYY-MM-DD" sqref="I1:I1048576 AE1:AE1048576" xr:uid="{87A554BA-43A4-4D4B-9158-4430D3C8FB3D}"/>
+  <dataValidations count="8">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A1048576">
+      <formula1>Help!$C$2:$C$7</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E1048576">
+      <formula1>Help!$B$1:$B$5</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1048576">
+      <formula1>Help!$D$2:$D$50</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2:N1048576">
+      <formula1>Help!$E$2:$E$8</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q2:Q1048576">
+      <formula1>Help!$F$2:$F$6</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T$1:T$1048576">
+      <formula1>Help!$G$2:$G$9</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U2:U1048576">
+      <formula1>Help!$H$2:$H$9</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="W2:W1048576 AA2:AA1048576">
+      <formula1>Help!$I$2:$I$38</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="8">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000000000000}">
-          <x14:formula1>
-            <xm:f>Help!$C$2:$C$7</xm:f>
-          </x14:formula1>
-          <xm:sqref>A2:A1048576</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000001000000}">
-          <x14:formula1>
-            <xm:f>Help!$B$1:$B$5</xm:f>
-          </x14:formula1>
-          <xm:sqref>E2:E1048576</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
-          <x14:formula1>
-            <xm:f>Help!$D$2:$D$50</xm:f>
-          </x14:formula1>
-          <xm:sqref>G2:G1048576</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000003000000}">
-          <x14:formula1>
-            <xm:f>Help!$E$2:$E$8</xm:f>
-          </x14:formula1>
-          <xm:sqref>O2:O1048576</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000004000000}">
-          <x14:formula1>
-            <xm:f>Help!$F$2:$F$6</xm:f>
-          </x14:formula1>
-          <xm:sqref>R2:R1048576</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000005000000}">
-          <x14:formula1>
-            <xm:f>Help!$G$2:$G$9</xm:f>
-          </x14:formula1>
-          <xm:sqref>U1:U1048576</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000006000000}">
-          <x14:formula1>
-            <xm:f>Help!$H$2:$H$9</xm:f>
-          </x14:formula1>
-          <xm:sqref>V2:V1048576</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000007000000}">
-          <x14:formula1>
-            <xm:f>Help!$I$2:$I$38</xm:f>
-          </x14:formula1>
-          <xm:sqref>AB2:AB1048576 X2:X1048576</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
+  <pageSetup paperSize="1" orientation="portrait"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:I50"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="17.44140625" customWidth="1"/>
-    <col min="2" max="2" width="16.109375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="8.88671875" style="1"/>
-    <col min="4" max="4" width="32.6640625" customWidth="1"/>
-    <col min="5" max="5" width="13.6640625" customWidth="1"/>
-    <col min="6" max="6" width="19.44140625" customWidth="1"/>
-    <col min="7" max="7" width="13.44140625" customWidth="1"/>
-    <col min="8" max="8" width="13.77734375" customWidth="1"/>
-    <col min="9" max="9" width="27.109375" customWidth="1"/>
-    <col min="12" max="12" width="8.88671875" customWidth="1"/>
+    <col min="1" max="1" width="17.5" customWidth="1"/>
+    <col min="2" max="2" width="16.1272727272727" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8.87272727272727" style="1"/>
+    <col min="4" max="4" width="32.6272727272727" customWidth="1"/>
+    <col min="5" max="5" width="13.6272727272727" customWidth="1"/>
+    <col min="6" max="6" width="19.5" customWidth="1"/>
+    <col min="7" max="7" width="13.5" customWidth="1"/>
+    <col min="8" max="8" width="13.7545454545455" customWidth="1"/>
+    <col min="9" max="9" width="27.1272727272727" customWidth="1"/>
+    <col min="12" max="12" width="8.87272727272727" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -1186,7 +1777,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="15.6" customHeight="1">
+    <row r="4" ht="15.6" customHeight="1" spans="1:9">
       <c r="A4" s="2" t="s">
         <v>49</v>
       </c>
@@ -1313,7 +1904,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="4:9">
       <c r="D9" t="s">
         <v>84</v>
       </c>
@@ -1327,7 +1918,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="4:9">
       <c r="D10" t="s">
         <v>88</v>
       </c>
@@ -1338,7 +1929,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="4:9">
       <c r="D11" t="s">
         <v>91</v>
       </c>
@@ -1346,7 +1937,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="4:9">
       <c r="D12" t="s">
         <v>93</v>
       </c>
@@ -1354,7 +1945,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="4:9">
       <c r="D13" t="s">
         <v>95</v>
       </c>
@@ -1362,7 +1953,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="4:9">
       <c r="D14" t="s">
         <v>97</v>
       </c>
@@ -1370,7 +1961,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="4:9">
       <c r="D15" t="s">
         <v>99</v>
       </c>
@@ -1378,7 +1969,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="4:9">
       <c r="D16" t="s">
         <v>101</v>
       </c>
@@ -1562,52 +2153,52 @@
         <v>146</v>
       </c>
     </row>
-    <row r="39" spans="4:9">
+    <row r="39" spans="4:4">
       <c r="D39" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="40" spans="4:9">
+    <row r="40" spans="4:4">
       <c r="D40" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="41" spans="4:9">
+    <row r="41" spans="4:4">
       <c r="D41" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="42" spans="4:9">
+    <row r="42" spans="4:4">
       <c r="D42" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="43" spans="4:9">
+    <row r="43" spans="4:4">
       <c r="D43" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="44" spans="4:9">
+    <row r="44" spans="4:4">
       <c r="D44" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="45" spans="4:9">
+    <row r="45" spans="4:4">
       <c r="D45" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="46" spans="4:9">
+    <row r="46" spans="4:4">
       <c r="D46" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="47" spans="4:9">
+    <row r="47" spans="4:4">
       <c r="D47" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="48" spans="4:9">
+    <row r="48" spans="4:4">
       <c r="D48" t="s">
         <v>156</v>
       </c>
@@ -1624,6 +2215,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait"/>
+  <pageSetup paperSize="1" orientation="portrait"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(bulk-upload): employee id in template, submit button, refresh user list
- Template: EmployeeId column after UserName/Password (column N); the
  dropdowns after it moved with their columns. Admin-API 3.12.0 makes
  Employee Id mandatory and unique.
- A chosen file is only checked (EmployeeId column present, not empty)
  and shows "N user(s) ready"; the upload starts on the new Submit
  button.
- The user list reloads after users are created and when going back.
  Back only asks to confirm when a checked file is still waiting.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/assets/bulkuser_excel_sheet.xlsx
+++ b/src/assets/bulkuser_excel_sheet.xlsx
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="160">
   <si>
     <t>Title</t>
   </si>
@@ -516,6 +516,9 @@
   </si>
   <si>
     <t>test_UAT</t>
+  </si>
+  <si>
+    <t>EmployeeId</t>
   </si>
 </sst>
 </file>
@@ -1514,7 +1517,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AD2"/>
+  <dimension ref="A1:AE2"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelRow="1"/>
   <cols>
     <col min="1" max="1" width="14.5" customWidth="1"/>
@@ -1528,23 +1531,24 @@
     <col min="9" max="9" width="21.1272727272727" style="5" customWidth="1"/>
     <col min="10" max="10" width="9.12727272727273" style="4" customWidth="1"/>
     <col min="11" max="13" width="25.3727272727273" customWidth="1"/>
-    <col min="14" max="14" width="24" customWidth="1"/>
-    <col min="15" max="15" width="24.7545454545455" style="4" customWidth="1"/>
-    <col min="16" max="16" width="11.8727272727273" customWidth="1"/>
-    <col min="17" max="17" width="20.6272727272727" customWidth="1"/>
-    <col min="18" max="18" width="20.1272727272727" customWidth="1"/>
-    <col min="19" max="19" width="20.7545454545455" customWidth="1"/>
-    <col min="20" max="20" width="20.3727272727273" customWidth="1"/>
-    <col min="21" max="21" width="16.7545454545455" customWidth="1"/>
-    <col min="22" max="24" width="28.8727272727273" customWidth="1"/>
-    <col min="25" max="25" width="21.6272727272727" style="4" customWidth="1"/>
-    <col min="26" max="26" width="35.6272727272727" customWidth="1"/>
-    <col min="27" max="28" width="28.8727272727273" customWidth="1"/>
-    <col min="29" max="29" width="28.8727272727273" style="4" customWidth="1"/>
-    <col min="30" max="30" width="21.1272727272727" style="5" customWidth="1"/>
+    <col min="14" max="14" width="20" customWidth="1"/>
+    <col min="15" max="15" width="24" customWidth="1"/>
+    <col min="16" max="16" width="24.7545454545455" style="4" customWidth="1"/>
+    <col min="17" max="17" width="11.8727272727273" customWidth="1"/>
+    <col min="18" max="18" width="20.6272727272727" customWidth="1"/>
+    <col min="19" max="19" width="20.1272727272727" customWidth="1"/>
+    <col min="20" max="20" width="20.7545454545455" customWidth="1"/>
+    <col min="21" max="21" width="20.3727272727273" customWidth="1"/>
+    <col min="22" max="22" width="16.7545454545455" customWidth="1"/>
+    <col min="23" max="25" width="28.8727272727273" customWidth="1"/>
+    <col min="26" max="26" width="21.6272727272727" style="4" customWidth="1"/>
+    <col min="27" max="27" width="35.6272727272727" customWidth="1"/>
+    <col min="28" max="29" width="28.8727272727273" customWidth="1"/>
+    <col min="30" max="30" width="28.8727272727273" style="4" customWidth="1"/>
+    <col min="31" max="31" width="21.1272727272727" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="3" customFormat="1" ht="23.5" spans="1:30">
+    <row r="1" s="3" customFormat="1" ht="23.5" spans="1:31">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -1584,55 +1588,58 @@
       <c r="M1" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="7" t="s">
+      <c r="N1" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="O1" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="11" t="s">
+      <c r="P1" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="7" t="s">
+      <c r="Q1" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="6" t="s">
+      <c r="R1" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="7" t="s">
+      <c r="S1" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="7" t="s">
+      <c r="T1" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="7" t="s">
+      <c r="U1" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="7" t="s">
+      <c r="V1" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="7" t="s">
+      <c r="W1" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="6" t="s">
+      <c r="X1" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="6" t="s">
+      <c r="Y1" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="11" t="s">
+      <c r="Z1" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="7" t="s">
+      <c r="AA1" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="6" t="s">
+      <c r="AB1" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="13" t="s">
+      <c r="AC1" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="11" t="s">
+      <c r="AD1" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="9" t="s">
+      <c r="AE1" s="9" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1650,19 +1657,19 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1048576">
       <formula1>Help!$D$2:$D$50</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N2:N1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O2:O1048576">
       <formula1>Help!$E$2:$E$8</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q2:Q1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="R2:R1048576">
       <formula1>Help!$F$2:$F$6</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T$1:T$1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U$1:U$1048576">
       <formula1>Help!$G$2:$G$9</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U2:U1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V2:V1048576">
       <formula1>Help!$H$2:$H$9</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="W2:W1048576 AA2:AA1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X2:X1048576 AB2:AB1048576">
       <formula1>Help!$I$2:$I$38</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>